<commit_message>
added new pads for spark
</commit_message>
<xml_diff>
--- a/library/connectors.xlsx
+++ b/library/connectors.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitProjects\elem_altium_db2\library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6E781A4-C258-4694-B480-38E8FF5363E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AE3E761-DC78-4972-B729-A3CC8726BED2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Connectors" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="513" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="519" uniqueCount="210">
   <si>
     <t>Part Number</t>
   </si>
@@ -654,6 +654,18 @@
   </si>
   <si>
     <t>con-ru-f-2</t>
+  </si>
+  <si>
+    <t>PAD200x150_HOLE</t>
+  </si>
+  <si>
+    <t>Hole 2mm x 1.5 mm</t>
+  </si>
+  <si>
+    <t>PAD260x100_SMD_HOLE</t>
+  </si>
+  <si>
+    <t>Pad_Hole 2.6mm x 1 mm</t>
   </si>
 </sst>
 </file>
@@ -844,14 +856,13 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="2" fillId="4" borderId="0" xfId="4" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="19">
     <cellStyle name="Accent 1 1" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -2181,7 +2192,7 @@
       <c r="E43" t="s">
         <v>203</v>
       </c>
-      <c r="F43" s="4" t="s">
+      <c r="F43" t="s">
         <v>204</v>
       </c>
     </row>
@@ -3020,7 +3031,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="30.7109375" customWidth="1"/>
@@ -3133,6 +3144,28 @@
         <v>192</v>
       </c>
     </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>207</v>
+      </c>
+      <c r="D9" t="s">
+        <v>183</v>
+      </c>
+      <c r="E9" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>209</v>
+      </c>
+      <c r="D10" t="s">
+        <v>183</v>
+      </c>
+      <c r="E10" t="s">
+        <v>208</v>
+      </c>
+    </row>
   </sheetData>
   <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
   <pageMargins left="0.70000000000000007" right="0.70000000000000007" top="0.75" bottom="0.75" header="0.51181102362204722" footer="0.51181102362204722"/>

</xml_diff>

<commit_message>
fixed rf lib, added hmc431, added rf connectors
</commit_message>
<xml_diff>
--- a/library/connectors.xlsx
+++ b/library/connectors.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitProjects\elem_altium_db2\library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AE3E761-DC78-4972-B729-A3CC8726BED2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAC2094C-B379-4E64-B42D-BAEB17AEFB76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Connectors" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="519" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="530" uniqueCount="213">
   <si>
     <t>Part Number</t>
   </si>
@@ -666,6 +666,15 @@
   </si>
   <si>
     <t>Pad_Hole 2.6mm x 1 mm</t>
+  </si>
+  <si>
+    <t>226990-1</t>
+  </si>
+  <si>
+    <t>901-10512-3</t>
+  </si>
+  <si>
+    <t>Amphenol</t>
   </si>
 </sst>
 </file>
@@ -856,13 +865,14 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="2" fillId="4" borderId="0" xfId="4" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="19">
     <cellStyle name="Accent 1 1" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -1321,7 +1331,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K43"/>
+  <dimension ref="A1:K45"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="35.28515625" style="1" customWidth="1"/>
@@ -2194,6 +2204,46 @@
       </c>
       <c r="F43" t="s">
         <v>204</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A44" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="B44" t="s">
+        <v>210</v>
+      </c>
+      <c r="C44" t="s">
+        <v>210</v>
+      </c>
+      <c r="D44" t="s">
+        <v>210</v>
+      </c>
+      <c r="E44">
+        <v>2269901</v>
+      </c>
+      <c r="F44" s="4" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A45" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="B45" t="s">
+        <v>211</v>
+      </c>
+      <c r="C45" t="s">
+        <v>211</v>
+      </c>
+      <c r="D45" t="s">
+        <v>211</v>
+      </c>
+      <c r="E45" t="s">
+        <v>211</v>
+      </c>
+      <c r="F45" s="4" t="s">
+        <v>212</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added MCU and DS connector
</commit_message>
<xml_diff>
--- a/library/connectors.xlsx
+++ b/library/connectors.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitProjects\elem_altium_db2\library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B73F4E68-3E97-45A5-B694-6A9E4B1E8EF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DA15EDF-8833-48AB-B3E1-05A760C8EAA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="536" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="542" uniqueCount="217">
   <si>
     <t>Part Number</t>
   </si>
@@ -681,6 +681,12 @@
   </si>
   <si>
     <t>Scondar</t>
+  </si>
+  <si>
+    <t>con-ru-m-36</t>
+  </si>
+  <si>
+    <t>DS1079-M36</t>
   </si>
 </sst>
 </file>
@@ -1336,7 +1342,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K46"/>
+  <dimension ref="A1:K47"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="35.28515625" style="1" customWidth="1"/>
@@ -2269,6 +2275,26 @@
       </c>
       <c r="F46" t="s">
         <v>214</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>216</v>
+      </c>
+      <c r="B47" t="s">
+        <v>216</v>
+      </c>
+      <c r="C47" t="s">
+        <v>216</v>
+      </c>
+      <c r="D47" t="s">
+        <v>215</v>
+      </c>
+      <c r="E47" t="s">
+        <v>216</v>
+      </c>
+      <c r="F47" s="1" t="s">
+        <v>47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added misc for spark and KPA
</commit_message>
<xml_diff>
--- a/library/connectors.xlsx
+++ b/library/connectors.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitProjects\elem_altium_db2\library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8043A1CB-AB81-4AFA-A46F-42EEC53A56F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BD4926A-36CC-4A0A-BF7B-57B8BD15BC04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Connectors" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="548" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="566" uniqueCount="226">
   <si>
     <t>Part Number</t>
   </si>
@@ -696,6 +696,24 @@
   </si>
   <si>
     <t>PLL-40</t>
+  </si>
+  <si>
+    <t>РПС1-37Ш</t>
+  </si>
+  <si>
+    <t>АСЛР.434410.022ТУ</t>
+  </si>
+  <si>
+    <t>РПС1-37Г</t>
+  </si>
+  <si>
+    <t>con-ru-m-37</t>
+  </si>
+  <si>
+    <t>con-ru-f-37</t>
+  </si>
+  <si>
+    <t>РПС1-15Г</t>
   </si>
 </sst>
 </file>
@@ -2743,7 +2761,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="30.5703125" customWidth="1"/>
@@ -3152,6 +3170,66 @@
       </c>
       <c r="F20" t="s">
         <v>176</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>220</v>
+      </c>
+      <c r="B21" t="s">
+        <v>220</v>
+      </c>
+      <c r="C21" t="s">
+        <v>220</v>
+      </c>
+      <c r="D21" t="s">
+        <v>223</v>
+      </c>
+      <c r="E21" t="s">
+        <v>220</v>
+      </c>
+      <c r="F21" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>222</v>
+      </c>
+      <c r="B22" t="s">
+        <v>222</v>
+      </c>
+      <c r="C22" t="s">
+        <v>222</v>
+      </c>
+      <c r="D22" t="s">
+        <v>224</v>
+      </c>
+      <c r="E22" t="s">
+        <v>222</v>
+      </c>
+      <c r="F22" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>225</v>
+      </c>
+      <c r="B23" t="s">
+        <v>225</v>
+      </c>
+      <c r="C23" t="s">
+        <v>225</v>
+      </c>
+      <c r="D23" t="s">
+        <v>113</v>
+      </c>
+      <c r="E23" t="s">
+        <v>225</v>
+      </c>
+      <c r="F23" t="s">
+        <v>221</v>
       </c>
     </row>
   </sheetData>

</xml_diff>